<commit_message>
Stage 2: RM cost on the part register
RM formulas move into master data (scopes rm_<family>); material rate and scrap value become
approved country rates in the rate library; each result is a numbered, traced RM cost version that
records the rate versions it used. New rates never change a stored cost (recalculate on purpose).
RM column, filters and per-variant roll-up on Parts and Dashboard, RM cost sheet in Excel and PDF,
and the Estimate page opens a registered part and saves back to it.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D29HjsuVEAxZgCF9RbbAEX
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Parameters" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Materials" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$F$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +43,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00102A43"/>
+        <fgColor rgb="000E1A2C"/>
       </patternFill>
     </fill>
   </fills>
@@ -480,6 +480,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Currency shown on cost results</t>
@@ -1827,15 +1828,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1856,16 +1855,6 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>rate_per_kg</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>scrap_rate_per_kg</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
           <t>notes</t>
         </is>
       </c>
@@ -1884,15 +1873,9 @@
       <c r="C2" t="n">
         <v>0.905</v>
       </c>
-      <c r="D2" t="n">
-        <v>110</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -1910,15 +1893,9 @@
       <c r="C3" t="n">
         <v>1.04</v>
       </c>
-      <c r="D3" t="n">
-        <v>180</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -1936,15 +1913,9 @@
       <c r="C4" t="n">
         <v>1.2</v>
       </c>
-      <c r="D4" t="n">
-        <v>260</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -1962,15 +1933,9 @@
       <c r="C5" t="n">
         <v>1.13</v>
       </c>
-      <c r="D5" t="n">
-        <v>230</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -1988,15 +1953,9 @@
       <c r="C6" t="n">
         <v>1.13</v>
       </c>
-      <c r="D6" t="n">
-        <v>250</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2014,15 +1973,9 @@
       <c r="C7" t="n">
         <v>1.36</v>
       </c>
-      <c r="D7" t="n">
-        <v>330</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2040,15 +1993,9 @@
       <c r="C8" t="n">
         <v>1.53</v>
       </c>
-      <c r="D8" t="n">
-        <v>300</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2066,15 +2013,9 @@
       <c r="C9" t="n">
         <v>1.41</v>
       </c>
-      <c r="D9" t="n">
-        <v>220</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2092,15 +2033,9 @@
       <c r="C10" t="n">
         <v>2.74</v>
       </c>
-      <c r="D10" t="n">
-        <v>260</v>
-      </c>
-      <c r="E10" t="n">
-        <v>180</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2118,15 +2053,9 @@
       <c r="C11" t="n">
         <v>2.71</v>
       </c>
-      <c r="D11" t="n">
-        <v>265</v>
-      </c>
-      <c r="E11" t="n">
-        <v>180</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2144,15 +2073,9 @@
       <c r="C12" t="n">
         <v>6.6</v>
       </c>
-      <c r="D12" t="n">
-        <v>300</v>
-      </c>
-      <c r="E12" t="n">
-        <v>220</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2170,15 +2093,9 @@
       <c r="C13" t="n">
         <v>1.81</v>
       </c>
-      <c r="D13" t="n">
-        <v>500</v>
-      </c>
-      <c r="E13" t="n">
-        <v>300</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2196,15 +2113,9 @@
       <c r="C14" t="n">
         <v>7.2</v>
       </c>
-      <c r="D14" t="n">
-        <v>45</v>
-      </c>
-      <c r="E14" t="n">
-        <v>40</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2222,15 +2133,9 @@
       <c r="C15" t="n">
         <v>7.1</v>
       </c>
-      <c r="D15" t="n">
-        <v>55</v>
-      </c>
-      <c r="E15" t="n">
-        <v>45</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2248,15 +2153,9 @@
       <c r="C16" t="n">
         <v>7.85</v>
       </c>
-      <c r="D16" t="n">
-        <v>65</v>
-      </c>
-      <c r="E16" t="n">
-        <v>50</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2274,15 +2173,9 @@
       <c r="C17" t="n">
         <v>2.68</v>
       </c>
-      <c r="D17" t="n">
-        <v>250</v>
-      </c>
-      <c r="E17" t="n">
-        <v>170</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2300,15 +2193,9 @@
       <c r="C18" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="D18" t="n">
-        <v>750</v>
-      </c>
-      <c r="E18" t="n">
-        <v>550</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2326,15 +2213,9 @@
       <c r="C19" t="n">
         <v>7.85</v>
       </c>
-      <c r="D19" t="n">
-        <v>65</v>
-      </c>
-      <c r="E19" t="n">
-        <v>30</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2352,15 +2233,9 @@
       <c r="C20" t="n">
         <v>7.85</v>
       </c>
-      <c r="D20" t="n">
-        <v>72</v>
-      </c>
-      <c r="E20" t="n">
-        <v>30</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2378,15 +2253,9 @@
       <c r="C21" t="n">
         <v>7.93</v>
       </c>
-      <c r="D21" t="n">
-        <v>230</v>
-      </c>
-      <c r="E21" t="n">
-        <v>110</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2404,15 +2273,9 @@
       <c r="C22" t="n">
         <v>2.68</v>
       </c>
-      <c r="D22" t="n">
-        <v>300</v>
-      </c>
-      <c r="E22" t="n">
-        <v>150</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
@@ -2430,20 +2293,14 @@
       <c r="C23" t="n">
         <v>8.960000000000001</v>
       </c>
-      <c r="D23" t="n">
-        <v>850</v>
-      </c>
-      <c r="E23" t="n">
-        <v>650</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Example rate - replace with your current price</t>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Density: typical value - check your datasheet. Rates: Rates page (material / material_scrap)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F23"/>
+  <autoFilter ref="A1:D23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Stage 8: part cost
Piece cost = RM + process (cycle x MHR of the machine the clamp force selects
+ operators x labour rate) + secondary operations + inserts + rejection +
overhead + profit + packing + tool amortisation + logistics, as Cost formulas
of the new scope piece with fully traced inputs (MHR and labour rate grafted
with their trace). Numbered part cost versions with an outdated flag, typed
cycle / cavities / secondary ops, Excel + PDF with full backup, and the Part
cost block on the part panel. Insert moulding: BOP price x quantity +
handling, loading time per shot, extra rejection and inserts lost.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JU1N3Zc31U18UVeHBq4Fes
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,13 +427,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="41" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -2012,8 +2012,181 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>operator_grade</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>operator</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Labour grade of the moulding / casting operator (Labour grades)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>operators_per_machine</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>persons</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Operators per machine (0.5 = one operator runs two machines)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>secondary_ops_pct</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>% of process</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Secondary operations (deburr, inspection, assembly) as % of the process cost; typed per part to override</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>rejection_pct</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Process rejection</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>die_casting</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>rejection_pct</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>4</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Process rejection (porosity, trimming)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>part_overhead_pct</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>5</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>% of conversion</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Admin / selling overhead on process + secondary cost (factory overhead is already in the MHR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>packing_pct</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Packing as % of the ex-works cost before packing</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E63"/>
+  <autoFilter ref="A1:E70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Stage 9: sheet-metal tools I
Operation sequence suggested from the 3D model (editable), progressive vs
multi-stage, stage weight, force per operation, tonnage with safety factor,
press selection and formability checks. Sheet materials, operations, rules and
checks are new tables in the mould & die database (EXAMPLE rows).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JU1N3Zc31U18UVeHBq4Fes
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,11 +427,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="41" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
@@ -2185,8 +2185,231 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>press_machine_process</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Machines process that takes sheet-metal press tonnage</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>stripping_pct</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>10</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>% of cutting</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Stripping force as % of the cutting force</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>progressive_min_volume</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>parts/yr</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Progressive die when the annual volume is at least this</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>progressive_max_len_mm</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>300</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Progressive die only up to this part length</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>progressive_max_draw_mm</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>15</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Progressive die only up to this draw depth (deeper: multi-stage / transfer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>default_bend_radius_factor</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>× t</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Inside bend radius assumed when the model has sharp corners</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>draw_height_ratio</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>5</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>× t</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>EXAMPLE: A part without bends taller than this × thickness is treated as drawn</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>bend_angle_deg</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>90</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>°</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Bend angle assumed for the springback estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>max_springback_deg</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>2</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>°</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Flag springback above this</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E70"/>
+  <autoFilter ref="A1:E79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Stage 10: sheet-metal tools II
Flat pattern (real outline for flat parts, developed rectangle for bent ones),
progressive strip layout from the new Strip rules (pitch, bridge, edge, width,
stations, pilots, utilisation, both feed directions), blank and strip DXF and a
PDF tool pack with dimensioned blank, strip layout and simplified stage sketches.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JU1N3Zc31U18UVeHBq4Fes
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2408,8 +2408,233 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>bridge_min_mm</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Smallest bridge between blanks in the strip</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>bridge_t_factor</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>× t</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Bridge as a multiple of thickness</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>edge_min_mm</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>2</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Smallest edge margin on each side of the strip</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>edge_t_factor</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>× t</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Edge margin as a multiple of thickness</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>carrier_mm</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Extra carrier width across the strip</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>idle_stations</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>stations</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Idle stations in the die (strength, clearance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>pilots</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Pilot holes per pitch</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>pilot_min_dia_mm</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>3</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Smallest pilot diameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>strip_max_width_mm</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>300</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Widest strip the line takes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E79"/>
+  <autoFilter ref="A1:E88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Stage 11: country comparison and landed cost in India
Part and tool made in each country with its approved rates, ex-works in local
currency / USD / INR, then freight, insurance, BCD by HS code and origin (FTA
switchable), SWS, IGST with credit shown apart, clearance and inland transport
-> landed cost in INR. Forex scenario, stacked bar chart, cheapest highlighted,
Excel + PDF. HS codes are master data; duty, freight and import rates are
approved rate-library versions (EXAMPLE seeds).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JU1N3Zc31U18UVeHBq4Fes
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2633,8 +2633,58 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>igst_claimable</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>1 = yes</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>EXAMPLE: 1 if the IGST paid on import is claimable as input credit (shown separately)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>fx_scenario_pct</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>5</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Forex scenario ± shown in the country comparison</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E88"/>
+  <autoFilter ref="A1:E90"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Stage 15: harness and PCB costing
Cost per harness / per board from a reviewed BOM extract: wires from the Part
library or copper content x (copper rate + conversion), parts from the Part
library, processing with MHR and labour, bare board from the rate library, then
rejection, overhead, profit and packing as Cost formulas. Traced, parts not in
the library listed as not priced, Excel + PDF.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JU1N3Zc31U18UVeHBq4Fes
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2683,8 +2683,33 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>pcb_panel_waste_pct</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>15</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Bare-board panel waste and set-up share added to the board cost</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E90"/>
+  <autoFilter ref="A1:E91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Stages 18 and 19: EPS (thermocole) moulding and PET stretch blow moulding
New part types eps and blow built into the existing stages: processes and
materials, RM families (foam weight; bottle shell weight from surface x wall),
aluminium tools with steam chests and blow-mould holders and their BOM rules,
EPS and ISBM machines, locking force from steam / blow pressure, steam and
preform conversion in the part cost, HS 3923 duty. All values are EXAMPLE rows.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JU1N3Zc31U18UVeHBq4Fes
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$91</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$D$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$134</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$D$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2708,8 +2708,1067 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>runner_pct</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>3</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Trim, flash and fines</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>process_loss_pct</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>4</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Start-up and reject loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>cycle_time_s</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>150</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>EXAMPLE: EPS moulding cycle: fill, steam, cooling, demould</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>oee_pct</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>70</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>EXAMPLE: OEE</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>max_cavities</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>4</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>cavities</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Blocks per chest</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>plate_length_mm</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Steam chest inner length</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>plate_width_mm</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Steam chest inner width</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>spacing_mm</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>40</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Spacing between blocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>tool_life_shots</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>300000</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>shots</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Aluminium tool life</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>standard_cavities</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 6, 8</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Allowed cavity counts</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>cycle_base_s</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>8</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Stage C rule: cycle = base + cooling factor x wall^2 (fill, open, eject time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>cooling_factor_s_per_mm2</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>2</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>s/mm2</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Stage C rule: cooling time per mm^2 of main wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>cavity_pressure_bar</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Steam pressure on the projected area</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>clamp_safety_factor</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Locking safety factor</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>trial_machine_process</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>EPS moulding</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Machine process used for try-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>trials</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>2</v>
+      </c>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Try-outs</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>trial_hours_each</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>6</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Hours per try-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>trial_shots_each</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>30</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>shots</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Shots per try-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>steam_kg_per_kg_part</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>kg/kg</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Steam per kg of moulded EPS (pre-expansion and moulding)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>rejection_pct</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>3</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Process rejection</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>runner_pct</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Preform gate and neck allowance</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>process_loss_pct</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Start-up and reject loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>cycle_time_s</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>6</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Cycle per shot of all cavities</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>oee_pct</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>80</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>EXAMPLE: OEE</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>max_cavities</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>8</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>cavities</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Cavities of the largest machine</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>plate_length_mm</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Mould area length</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>plate_width_mm</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>800</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Mould area width</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>spacing_mm</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>40</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Spacing between cavities</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>tool_life_shots</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>shots</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Blow mould life</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>standard_cavities</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>1, 2, 4, 6, 8, 10, 12, 16</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Allowed cavity counts</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>cycle_base_s</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>8</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Stage C rule: cycle = base + cooling factor x wall^2 (fill, open, eject time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>cooling_factor_s_per_mm2</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>2</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>s/mm2</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Stage C rule: cooling time per mm^2 of main wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>cavity_pressure_bar</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>35</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Blow pressure on the projected area</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>clamp_safety_factor</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Locking safety factor</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>trial_machine_process</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Stretch blow moulding</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Machine process used for try-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>trials</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>3</v>
+      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Try-outs</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>trial_hours_each</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>4</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Hours per try-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>trial_shots_each</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>500</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>shots</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Shots per try-out</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>blow_wall_mm</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Average bottle wall (weight = outer surface x wall x density)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>preform_conversion_pct</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>28</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>% of resin</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Preform injection moulding conversion (machine, labour, tool, margin) as % of resin cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>rejection_pct</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>2</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Process rejection</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>steam_kg_per_kg_part</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>kg/kg</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Steam per kg of moulded part (EPS only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>preform_conversion_pct</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>% of resin</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>EXAMPLE: Preform conversion (bottles only)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E91"/>
+  <autoFilter ref="A1:E134"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2720,11 +3779,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
   </cols>
@@ -3191,8 +4250,108 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>EPS bead grade S (20 kg/m3)</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>EXAMPLE density. Foamed part density. Rates: Rates page (material / material_scrap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>EPS bead grade F, flame retardant (25 kg/m3)</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>EXAMPLE density. Foamed part density. Rates: Rates page (material / material_scrap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PET bottle grade (IV 0.80)</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>EXAMPLE density. Resin density, used for the shell weight. Rates: Rates page (material / material_scrap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>blow</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>rPET food grade</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>EXAMPLE density. Resin density. Rates: Rates page (material / material_scrap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>plastic</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PET preform grade</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>EXAMPLE density. For preform injection moulding. Rates: Rates page (material / material_scrap)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D23"/>
+  <autoFilter ref="A1:D28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Stage 20: capacity 0-3000 t, 3D design correction, stage-wise sheet-metal tool design, design pack downloads
- Machines, mould bases / die holders and machine rates up to 3000 t (capacity_db), validation page Capacity & tools
- Draft correction on the 3D model from the simulation, mould concept in 3D
- Stage tool rules (master data), stage-wise sheet-metal die sets in 3D with press selection by tonnage and bolster
- Design pack: Excel, PDF, PowerPoint, 3D report (HTML + STEP), corrected drawing (PDF, DXF), simulation video (MP4)
- Free-software registry and install notes; tests, README, ROADMAP

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xeoqohm56cQdFVh2rYc1k5
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$134</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$135</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$D$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E134"/>
+  <dimension ref="A1:E135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3767,8 +3767,33 @@
         </is>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>later_draw_ratio</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Reduction ratio of every draw after the first (EXAMPLE)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E134"/>
+  <autoFilter ref="A1:E135"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Stage 20 completion: real forming surfaces, true core/cavity split, sheet-metal model correction, FEA, cycle-time fix
- Wall thickness by cone rays, wall ends ignored, area-weighted percentiles (cover cycle 1000 s -> 18 s)
- Core/cavity split by the part's envelopes; slide/lifter proposals as markers
- Forming die and punch cut from the part for the last forming stage; springback overbend rule
- Sheet-metal correction: bend radii and minimum holes on the 3D model, stage design on the corrected part
- Structural check with Gmsh + CalculiX (insert and die block), VTK output for ParaView
- Tests and README updated

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xeoqohm56cQdFVh2rYc1k5
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$135</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$150</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$D$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E135"/>
+  <dimension ref="A1:E150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3792,8 +3792,371 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>plastic</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>fea_e_mpa</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>210000</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Young's modulus of tool steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>plastic</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>fea_poisson</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Poisson's ratio of tool steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>plastic</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>fea_yield_mpa</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>800</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Yield strength of the insert steel (EXAMPLE: pre-hardened P20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>plastic</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>fea_safety</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Safety factor on yield</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>plastic</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>fea_max_deflection_mm</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Allowed elastic deflection of an insert or die block</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>die_casting</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>fea_e_mpa</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>210000</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Young's modulus of tool steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>die_casting</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>fea_poisson</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Poisson's ratio of tool steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>die_casting</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>fea_yield_mpa</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>800</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Yield strength of the insert steel (EXAMPLE: pre-hardened P20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>die_casting</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>fea_safety</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Safety factor on yield</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>die_casting</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>fea_max_deflection_mm</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Allowed elastic deflection of an insert or die block</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>fea_e_mpa</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>210000</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Young's modulus of tool steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>fea_poisson</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Poisson's ratio of tool steel</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>fea_yield_mpa</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>800</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Yield strength of the insert steel (EXAMPLE: pre-hardened P20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>fea_safety</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Safety factor on yield</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>fea_max_deflection_mm</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Allowed elastic deflection of an insert or die block</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E135"/>
+  <autoFilter ref="A1:E150"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Stage 23: progressive vs stage-die comparison for sheet metal with full drawing package
Both die types get a full production design; comparison of press tonnage, gross raw material and strip layout, process cost, tool cost and cost per part with break-even; Excel, PDF and package ZIP; Progressive vs stage tab on the tool-design page.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xeoqohm56cQdFVh2rYc1k5
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$155</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$D$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E150"/>
+  <dimension ref="A1:E155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4155,8 +4155,133 @@
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>spm_progressive</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>60</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>strokes/min</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Strokes per minute of the progressive die</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>spm_stage</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>25</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>parts/min</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Parts per minute of one stage die (feeding by hand or robot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>operators_stage_press</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>1</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>persons</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Operators per press in a stage line (progressive uses operators_per_machine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>scrap_credit_pct</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>40</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Scrap sold at this % of the material rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>tool_markup_pct</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>25</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Toolroom design, try-out, overhead and margin on the tool made-parts cost</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E150"/>
+  <autoFilter ref="A1:E155"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Large parts (10-20 kg, up to 4000 t) and tool-design audit gaps closed
Machines to 4000 t / presses to 3000 t / HPDC 2500 t, made-to-order bases and heavy die sets,
large sheet, bed-size check, drawn-part detection, draw / trim / U-bend dies, mould gating,
slides, lifters, hot runner, die-casting, EPS and blow features, foundry tool cost and pattern
design, EPS / blow / foundry simulation, draft correction, large samples, re-audit PDF, tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015t1hrgzuZh9SofBRJTHBCo
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -480,7 +480,6 @@
           <t>INR</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Currency shown on cost results</t>
@@ -1832,7 +1831,6 @@
           <t>Injection moulding</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
           <t>Stage 4 try-out: process name of the machines (Machines sheet) the try-out machine is chosen from</t>
@@ -1930,7 +1928,6 @@
           <t>Die casting</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>Stage 4 try-out: process name of the machines (Machines sheet) the try-out machine is chosen from</t>
@@ -2028,7 +2025,6 @@
           <t>operator</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
           <t>EXAMPLE: Labour grade of the moulding / casting operator (Labour grades)</t>
@@ -2201,7 +2197,6 @@
           <t>Press</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
           <t>EXAMPLE: Machines process that takes sheet-metal press tonnage</t>
@@ -2949,7 +2944,6 @@
           <t>1, 2, 3, 4, 6, 8</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr">
         <is>
           <t>EXAMPLE: Allowed cavity counts</t>
@@ -3072,7 +3066,6 @@
           <t>EPS moulding</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr">
         <is>
           <t>EXAMPLE: Machine process used for try-out</t>
@@ -3093,7 +3086,6 @@
       <c r="C107" t="n">
         <v>2</v>
       </c>
-      <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
         <is>
           <t>EXAMPLE: Try-outs</t>
@@ -3441,7 +3433,6 @@
           <t>1, 2, 4, 6, 8, 10, 12, 16</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr">
         <is>
           <t>EXAMPLE: Allowed cavity counts</t>
@@ -3564,7 +3555,6 @@
           <t>Stretch blow moulding</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
           <t>EXAMPLE: Machine process used for try-out</t>
@@ -3585,7 +3575,6 @@
       <c r="C127" t="n">
         <v>3</v>
       </c>
-      <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr">
         <is>
           <t>EXAMPLE: Try-outs</t>
@@ -3783,7 +3772,6 @@
           <t>Press</t>
         </is>
       </c>
-      <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr">
         <is>
           <t>EXAMPLE: Stage 23 try-out of dies: process name of the presses (Machines)</t>
@@ -3862,6 +3850,193 @@
       <c r="E138" t="inlineStr">
         <is>
           <t>EXAMPLE: Stage 23 strokes per try-out (material)</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>large_sheet_length_mm</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>EXAMPLE: sheet / cut-to-length coil used when the blank does not fit the standard sheet (large parts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>large_sheet_width_mm</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>EXAMPLE: widest sheet / coil for large blanks</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>foundry</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>cavity_pressure_bar</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>0</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>EXAMPLE: no clamp force for sand moulds (pattern equipment)</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>foundry</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>clamp_safety_factor</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>1</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>EXAMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>foundry</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>trial_machine_process</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Foundry moulding</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>EXAMPLE: machine used for the pattern trial</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>foundry</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>trials</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>1</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>EXAMPLE: pattern trials</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>foundry</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>trial_hours_each</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>4</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>EXAMPLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>foundry</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>trial_shots_each</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>10</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>moulds</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>EXAMPLE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stage 41: progressive die vs stage dies; part cost amortised over tool / mould life
- Sheet-metal part page: both die types costed live (scope sheet_compare): time per part, presses,
  operators, process cost, die set cost, die life, die sets, tool CAPEX, amortisation, part cost,
  cheaper die type with INR saving per part and year, break-even volume (search over 0.1x-10x volume)
- Part cost amortisation = one tool / min(tool_life_shots x cavities, programme / tools for capacity)
  (the one shipped piece row changed, approved); machined fixture life added (EXAMPLE)
- New Parameters, Cost formulas and Formula inputs only added (EXAMPLE); fingerprints rebuilt
- Ask AI can read the comparison; README section, ROADMAP row 41, project memory

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xeoqohm56cQdFVh2rYc1k5
</commit_message>
<xml_diff>
--- a/master_data/master_data.xlsx
+++ b/master_data/master_data.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameters'!$A$1:$E$177</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materials'!$A$1:$F$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,11 +427,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E167"/>
+  <dimension ref="A1:E177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="41" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
@@ -4568,8 +4568,258 @@
         </is>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>stage_hit_time_s</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>6</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>EXAMPLE: one press hit with manual loading per stage die (stage 41 comparison)</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>stage_operators_per_press</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>1</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>operators</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>EXAMPLE: operators per press for stage dies (manual load / unload)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>progressive_spm</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>30</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>strokes/min</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>EXAMPLE: strokes per minute of a coil-fed progressive die</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>progressive_operators</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>operators</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>EXAMPLE: operators per progressive press (coil fed, one operator for two presses)</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>stage_die_life_strokes</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>strokes</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>EXAMPLE: life of a stage die before replacement (one stroke per part)</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>progressive_die_life_strokes</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>strokes</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>EXAMPLE: life of a progressive die before replacement (one stroke per part)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>compare_volume_min_factor</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>× volume</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>EXAMPLE: break-even chart from this share of the part's annual volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>compare_volume_max_factor</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>10</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>× volume</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>EXAMPLE: break-even chart up to this multiple of the part's annual volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>sheet_metal</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>compare_volume_points</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>9</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>points</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>EXAMPLE: volumes in the break-even table (spread evenly on a log scale)</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>machined</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>tool_life_shots</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>500000</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>parts</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>EXAMPLE: fixture life in parts before it is replaced (tool amortisation, stage 41)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E167"/>
+  <autoFilter ref="A1:E177"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>